<commit_message>
Filter deals: drop sub-$20M raises and India/Kenya; brief descriptions
Apply >$20M floor to funding rounds (M&A any size); exclude India (WeRize)
and Kenya (Sumac); also drop sub-$20M raises Cense, Harmoney, Aveni.
Rewrite Target Description as a single brief company sentence with no
round-size/EV metadata. 24 -> 19 rows. Regenerate xlsx and csv.
</commit_message>
<xml_diff>
--- a/fintech-deals-verified.xlsx
+++ b/fintech-deals-verified.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Verified Deals Jun 2026" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Verified Deals Jun 2026'!$A$1:$K$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Verified Deals Jun 2026'!$A$1:$K$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -457,7 +457,7 @@
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="60" customWidth="1" min="10" max="10"/>
+    <col width="55" customWidth="1" min="10" max="10"/>
     <col width="48" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
@@ -556,7 +556,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Integrated insurance distribution + RIA advisory network serving agents/advisors across 700+ US cities; deal ~$9.6M incl. cash, stock and earnout.</t>
+          <t>A US insurance-distribution and registered-investment-advisory network.</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -601,7 +601,7 @@
       <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Loan-servicing technology for non-bank lenders; ~A$55bn AUA across the full loan lifecycle. Perpetual took an initial 70% stake.</t>
+          <t>An Australian loan-servicing technology provider for non-bank lenders.</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -646,7 +646,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Core &amp; digital banking software (Phoenix Core System, Malauzai Digital Banking, Fusion Analytics) used by hundreds of US banks/credit unions.</t>
+          <t>Finastra's US core and digital banking software unit (Phoenix, Malauzai).</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -663,27 +663,27 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Kenya</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Strategic M&amp;A</t>
+          <t>Capital Raise</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Sumac Microfinance Bank</t>
+          <t>Capchase</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Moniepoint</t>
+          <t>01 Advisors (lead)</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
@@ -691,44 +691,44 @@
       <c r="I5" s="2" t="inlineStr"/>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Kenyan microfinance bank (78% stake acquired) marking Moniepoint's entry into East Africa. NOTE: announced/closed late MARCH 2026, not June.</t>
+          <t>A US provider of non-dilutive, revenue-based financing for B2B software firms.</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>https://www.businesswire.com/news/home/20260331855947/en/Moniepoint-Inc.-Enters-Kenyan-Market-With-Acquisition-of-Sumac-Microfinance-Bank</t>
+          <t>https://news.crunchbase.com/venture/fintech-capchase-b2b-bnpl-200m-debt-equity/</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Banking &amp; Lending Tech</t>
+          <t>Capital Markets Tech</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Capital Raise</t>
+          <t>Strategic M&amp;A</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Capchase</t>
+          <t>Funded Trading Plus</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>01 Advisors (lead)</t>
+          <t>Instant Funding</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -736,24 +736,24 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>B2B / vendor financing platform ('Affirm for B2B'). Raised $26M equity + $174M credit facility.</t>
+          <t>A UK proprietary trading firm offering funded-trader evaluation accounts.</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>https://news.crunchbase.com/venture/fintech-capchase-b2b-bnpl-200m-debt-equity/</t>
+          <t>https://windsordrake.com/market-intelligence/transactions/funded-trading-plus-instant-funding-2026</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Banking &amp; Lending Tech</t>
+          <t>Corporate Financial Function</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -768,12 +768,12 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>WeRize</t>
+          <t>Ramp</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Sony Innovation Fund (lead)</t>
+          <t>ICONIQ, GIC, Ontario Teachers' (lead)</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
@@ -781,29 +781,29 @@
       <c r="I7" s="2" t="inlineStr"/>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>AI-powered credit, insurance and investment platform for small-city ('Bharat') India. Raised $7M pre-Series C.</t>
+          <t>A US corporate spend-management and financial-operations platform.</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>https://inc42.com/buzz/fintech-startup-werize-raises-7-mn-to-expand-product-offerings/</t>
+          <t>https://www.prnewswire.com/news-releases/ramp-raises-series-f-at-44-billion-valuation-302791103.html</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Capital Markets Tech</t>
+          <t>Corporate Financial Function</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Capital Raise</t>
+          <t>Strategic M&amp;A</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -813,12 +813,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Cense</t>
+          <t>Leapfin</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>G+D Ventures &amp; Rabo Investments (co-lead)</t>
+          <t>Airwallex</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
@@ -826,44 +826,44 @@
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Digital-asset compliance &amp; evidence platform for banks/financial institutions. Raised EUR 6.5M seed. (Closer to RegTech / Financial Info than Capital Markets.)</t>
+          <t>A US revenue-recognition and accounting-automation software provider.</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>https://fintech.global/2026/06/04/cense-raises-e6-5m-seed-round-for-digital-asset-compliance/</t>
+          <t>https://www.airwallex.com/global/newsroom/airwallex-acquires-leapfin-expanding-financial-lifecycle-capabilities</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Capital Markets Tech</t>
+          <t>Corporate Financial Function</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Strategic M&amp;A</t>
+          <t>Capital Raise</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Funded Trading Plus</t>
+          <t>Pivot</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Instant Funding</t>
+          <t>Forestay Capital &amp; Notion Capital (lead)</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
@@ -871,19 +871,19 @@
       <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Proprietary trading firm offering funded-trader evaluation products and funded trading accounts.</t>
+          <t>A French AI procurement and spend-management software provider.</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>https://windsordrake.com/market-intelligence/transactions/funded-trading-plus-instant-funding-2026</t>
+          <t>https://www.globenewswire.com/news-release/2026/05/21/3299278/0/en/Pivot-Raises-40-Million-Series-B-to-Replace-Legacy-Procurement-Software-with-an-Enterprise-AI-Operating-System.html</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Corporate Financial Function</t>
+          <t>Financial Info &amp; Analytics</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -898,17 +898,17 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Ramp</t>
+          <t>AlphaSense</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>ICONIQ, GIC, Ontario Teachers' (lead)</t>
+          <t>Vitruvian Partners, Accenture Ventures, J.P. Morgan Asset Mgmt (lead)</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -916,19 +916,19 @@
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>AI spend-management / financial-operations platform (corporate cards, expense, AP, treasury). Raised $750M Series F at $44B valuation.</t>
+          <t>A US AI-powered market-intelligence and research platform.</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/ramp-raises-series-f-at-44-billion-valuation-302791103.html</t>
+          <t>https://www.globenewswire.com/news-release/2026/06/03/3305968/0/en/alphasense-raises-350m-at-7-5b-valuation-and-surpasses-600m-in-annual-recurring-revenue.html</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Corporate Financial Function</t>
+          <t>Financial Info &amp; Analytics</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -948,12 +948,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Leapfin</t>
+          <t>PEER DATA</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Airwallex</t>
+          <t>Lukka</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
@@ -961,24 +961,24 @@
       <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Revenue-recognition &amp; reconciliation automation platform (record-to-report; GAAP/IFRS-ready financials).</t>
+          <t>A provider of data-provenance and compliance infrastructure for digital assets.</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>https://www.airwallex.com/global/newsroom/airwallex-acquires-leapfin-expanding-financial-lifecycle-capabilities</t>
+          <t>http://www.prnewswire.com/news-releases/lukka-acquires-peer-data-to-build-the-institutional-control-layer-for-digital-assets-and-data-commerce-302791630.html</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Corporate Financial Function</t>
+          <t>InsurTech</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -988,17 +988,17 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Pivot</t>
+          <t>Honeycomb Insurance</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Forestay Capital &amp; Notion Capital (lead)</t>
+          <t>Zeev Ventures (lead)</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
@@ -1006,24 +1006,24 @@
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>AI enterprise procurement / spend operating system (Paris-based). Raised $40M Series B. NOTE: source data listed US — company is French.</t>
+          <t>A US AI-driven commercial-property insurance underwriter.</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2026/05/21/3299278/0/en/Pivot-Raises-40-Million-Series-B-to-Replace-Legacy-Procurement-Software-with-an-Enterprise-AI-Operating-System.html</t>
+          <t>https://fortune.com/2026/06/04/honeycomb-insurance-ai-apartments-40-million/</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Corporate Financial Function</t>
+          <t>InsurTech</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1033,17 +1033,17 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Harmoney</t>
+          <t>Corgi</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Smile Sail</t>
+          <t>TCV (lead)</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
@@ -1051,19 +1051,19 @@
       <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>KYC/AML/counterparty-risk compliance orchestration platform (Ghent). EUR 10M strategic minority investment. (RegTech.)</t>
+          <t>A US full-stack commercial insurance platform.</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>https://fintech.global/2026/05/26/harmoney-eyes-european-growth-with-e10m-investment/</t>
+          <t>https://techcrunch.com/2026/05/28/corgi-announces-106m-raise-at-2-6b-valuation-three-weeks-after-160m-series-b/</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Financial Info &amp; Analytics</t>
+          <t>InsurTech</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1073,47 +1073,49 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Capital Raise</t>
+          <t>Strategic M&amp;A</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>AlphaSense</t>
+          <t>Aggne (Aggne Global)</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Vitruvian Partners, Accenture Ventures, J.P. Morgan Asset Mgmt (lead)</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr"/>
+          <t>Wipro</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>28.5</v>
+      </c>
       <c r="H14" s="2" t="inlineStr"/>
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>AI market-intelligence / research &amp; workflow platform. Raised $350M at $7.5B valuation; &gt;$600M ARR.</t>
+          <t>A US property-and-casualty insurance technology and consulting firm.</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2026/06/03/3305968/0/en/alphasense-raises-350m-at-7-5b-valuation-and-surpasses-600m-in-annual-recurring-revenue.html</t>
+          <t>https://www.business-standard.com/amp/companies/news/wipro-raises-stake-in-insurance-tech-firm-aggne-to-80-for-28-5-million-126060102064_1.html</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Financial Info &amp; Analytics</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1123,62 +1125,64 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>PEER DATA</t>
+          <t>KUBRA (Kubra Data Transfer)</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Lukka</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr"/>
+          <t>REPAY</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>372</v>
+      </c>
       <c r="H15" s="2" t="inlineStr"/>
       <c r="I15" s="2" t="inlineStr"/>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>Data provenance / Data Book of Record (DBOR) and compliance platform for institutional digital assets.</t>
+          <t>A Canadian billing and customer-payments technology provider for utilities and government.</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>http://www.prnewswire.com/news-releases/lukka-acquires-peer-data-to-build-the-institutional-control-layer-for-digital-assets-and-data-commerce-302791630.html</t>
+          <t>https://investors.repay.com/news-releases/news-release-details/repay-announces-agreement-acquire-kubra</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Financial Info &amp; Analytics</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Capital Raise</t>
+          <t>Strategic M&amp;A</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Aveni</t>
+          <t>Fee Navigator</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>PXN Ventures (lead)</t>
+          <t>NMI</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr"/>
@@ -1186,114 +1190,118 @@
       <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>AI compliance / assurance platform for financial services (Edinburgh). Raised GBP 12M.</t>
+          <t>A US AI merchant-pricing intelligence provider for payments.</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>https://fintech.global/2026/06/04/lloyds-and-nationwide-backed-aveni-raises-12m/</t>
+          <t>https://www.businesswire.com/news/home/20260602447713/en/NMI-Acquires-Fee-Navigator-Adding-AI-Powered-Pricing-Intelligence-to-Its-Embedded-Payments-Platform</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>InsurTech</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Capital Raise</t>
+          <t>SPAC merger (de-SPAC)</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Honeycomb Insurance</t>
+          <t>OpenPayd</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Zeev Ventures (lead)</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr"/>
+          <t>Titan Acquisition Corp (SPAC)</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>1100</v>
+      </c>
       <c r="H17" s="2" t="inlineStr"/>
       <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>AI underwriting platform for commercial property / real-estate (multifamily) insurance. Raised $40M.</t>
+          <t>A UK embedded-finance and payments-orchestration platform.</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>https://fortune.com/2026/06/04/honeycomb-insurance-ai-apartments-40-million/</t>
+          <t>https://www.globenewswire.com/news-release/2026/06/01/3304275/0/en/OpenPayd-Targets-Nasdaq-Listing-at-Unicorn-Valuation.html</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>InsurTech</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Capital Raise</t>
+          <t>Strategic M&amp;A</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Corgi</t>
+          <t>WonderFi</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>TCV (lead)</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr"/>
+          <t>Robinhood</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>182</v>
+      </c>
       <c r="H18" s="2" t="inlineStr"/>
       <c r="I18" s="2" t="inlineStr"/>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Full-stack commercial insurance platform. Raised $106M Series B1 at $2.6B valuation (3 weeks after a $160M Series B).</t>
+          <t>A Canadian operator of regulated crypto exchanges (Bitbuy and Coinsquare).</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>https://techcrunch.com/2026/05/28/corgi-announces-106m-raise-at-2-6b-valuation-three-weeks-after-160m-series-b/</t>
+          <t>https://www.newsfilecorp.com/release/299681/Robinhood-Completes-Acquisition-of-WonderFi</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>InsurTech</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1303,39 +1311,37 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Aggne (Aggne Global)</t>
+          <t>Absolute Payment Solutions</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Wipro</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="n">
-        <v>28.5</v>
-      </c>
+          <t>XFolio AI</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr"/>
       <c r="H19" s="2" t="inlineStr"/>
       <c r="I19" s="2" t="inlineStr"/>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>P&amp;C insurance technology / consulting services. Wipro raised its stake from 60% to 80% for $28.5M.</t>
+          <t>A UK Pay.UK-accredited Bacs payments service provider.</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>https://www.business-standard.com/amp/companies/news/wipro-raises-stake-in-insurance-tech-firm-aggne-to-80-for-28-5-million-126060102064_1.html</t>
+          <t>https://www.fintechfutures.com/m-a/xfolio-ai-acquires-absolute-payments-solutions</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>Real Estate &amp; Mortgage Tech</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1350,266 +1356,35 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>KUBRA (Kubra Data Transfer)</t>
+          <t>Accepted Financial Corp</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>REPAY</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="n">
-        <v>372</v>
-      </c>
+          <t>Shelter Lending Corporation</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr"/>
       <c r="H20" s="2" t="inlineStr"/>
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>Customer-experience billing &amp; payments technology for utilities/government. Announced 30 Mar 2026 (closed 1 Jun). Mississauga, Canada-based.</t>
+          <t>A Western-Canada alternative mortgage lender and brokerage.</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>https://investors.repay.com/news-releases/news-release-details/repay-announces-agreement-acquire-kubra</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Payments</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>Strategic M&amp;A</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-02</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>Fee Navigator</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>NMI</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr"/>
-      <c r="H21" s="2" t="inlineStr"/>
-      <c r="I21" s="2" t="inlineStr"/>
-      <c r="J21" s="2" t="inlineStr">
-        <is>
-          <t>AI merchant-pricing intelligence (analyzes merchant statements to recommend optimized pricing).</t>
-        </is>
-      </c>
-      <c r="K21" s="2" t="inlineStr">
-        <is>
-          <t>https://www.businesswire.com/news/home/20260602447713/en/NMI-Acquires-Fee-Navigator-Adding-AI-Powered-Pricing-Intelligence-to-Its-Embedded-Payments-Platform</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Payments</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>United Kingdom</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>SPAC merger (de-SPAC)</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>OpenPayd</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>Titan Acquisition Corp (SPAC)</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="n">
-        <v>1100</v>
-      </c>
-      <c r="H22" s="2" t="inlineStr"/>
-      <c r="I22" s="2" t="inlineStr"/>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>Embedded finance / fiat &amp; stablecoin payment orchestration. Nasdaq listing via SPAC at ~$1.1B equity value (NOT a strategic acquisition).</t>
-        </is>
-      </c>
-      <c r="K22" s="2" t="inlineStr">
-        <is>
-          <t>https://www.globenewswire.com/news-release/2026/06/01/3304275/0/en/OpenPayd-Targets-Nasdaq-Listing-at-Unicorn-Valuation.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>Payments</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Canada</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>Strategic M&amp;A (closed; announced 2025)</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>WonderFi</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>Robinhood</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="n">
-        <v>182</v>
-      </c>
-      <c r="H23" s="2" t="inlineStr"/>
-      <c r="I23" s="2" t="inlineStr"/>
-      <c r="J23" s="2" t="inlineStr">
-        <is>
-          <t>Canadian regulated crypto exchanges (Bitbuy, Coinsquare). ~C$250M (~US$182M). NOTE: announced 2025; 1 Jun = CLOSE, not announcement. Crypto exchange (arguably Capital Markets).</t>
-        </is>
-      </c>
-      <c r="K23" s="2" t="inlineStr">
-        <is>
-          <t>https://www.newsfilecorp.com/release/299681/Robinhood-Completes-Acquisition-of-WonderFi</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>Payments</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>United Kingdom</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Strategic M&amp;A</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-02</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>Absolute Payment Solutions</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>XFolio AI</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr"/>
-      <c r="H24" s="2" t="inlineStr"/>
-      <c r="I24" s="2" t="inlineStr"/>
-      <c r="J24" s="2" t="inlineStr">
-        <is>
-          <t>Pay.UK-accredited Bacs service provider; combined with XFolio AI (Paris) treasury &amp; payments platform.</t>
-        </is>
-      </c>
-      <c r="K24" s="2" t="inlineStr">
-        <is>
-          <t>https://www.fintechfutures.com/m-a/xfolio-ai-acquires-absolute-payments-solutions</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>Real Estate &amp; Mortgage Tech</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Canada</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>Strategic M&amp;A</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-20</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>Accepted Financial Corp</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>Shelter Lending Corporation</t>
-        </is>
-      </c>
-      <c r="G25" s="2" t="inlineStr"/>
-      <c r="H25" s="2" t="inlineStr"/>
-      <c r="I25" s="2" t="inlineStr"/>
-      <c r="J25" s="2" t="inlineStr">
-        <is>
-          <t>Western-Canada alternative mortgage lender/broker (Langley, BC). Services business rather than pure tech.</t>
-        </is>
-      </c>
-      <c r="K25" s="2" t="inlineStr">
-        <is>
           <t>https://www.cantechletter.com/newswires/shelter-lending-corporation-announces-acquisition-of-accepted-financial-corp-accelerating-national-growth-strategy/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K25"/>
+  <autoFilter ref="A1:K20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Split deals into two sheets: Growth Raises and Acquisitions
Growth Raises tab (6 rows): Sector, Target Country, Date, Target, Lead
Investor(s), Amount ($M), Valuation ($M), EV/Revenue, EV/EBITDA,
Description, Link. Acquisitions tab (13 rows) keeps Deal Type/Acquirer/EV.
Replace combined CSV with two split CSVs.
</commit_message>
<xml_diff>
--- a/fintech-deals-verified.xlsx
+++ b/fintech-deals-verified.xlsx
@@ -7,10 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Verified Deals Jun 2026" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Growth Raises" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Acquisitions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Verified Deals Jun 2026'!$A$1:$K$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Growth Raises'!$A$1:$K$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Acquisitions'!$A$1:$K$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -445,20 +447,369 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="50" customWidth="1" min="10" max="10"/>
+    <col width="46" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Target Country</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Lead Investor(s)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Amount ($M)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Valuation ($M)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>EV / Revenue</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>EV / EBITDA</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Target Description</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Link / Press Release</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Banking &amp; Lending Tech</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Capchase</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>01 Advisors</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>A US provider of non-dilutive, revenue-based financing for B2B software firms.</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>https://news.crunchbase.com/venture/fintech-capchase-b2b-bnpl-200m-debt-equity/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Corporate Financial Function</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Ramp</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>ICONIQ, GIC, Ontario Teachers'</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>750</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>44000</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>A US corporate spend-management and financial-operations platform.</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/ramp-raises-series-f-at-44-billion-valuation-302791103.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Corporate Financial Function</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Pivot</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Forestay Capital &amp; Notion Capital</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>A French AI procurement and spend-management software provider.</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.globenewswire.com/news-release/2026/05/21/3299278/0/en/Pivot-Raises-40-Million-Series-B-to-Replace-Legacy-Procurement-Software-with-an-Enterprise-AI-Operating-System.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Financial Info &amp; Analytics</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>AlphaSense</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Vitruvian Partners, Accenture Ventures, J.P. Morgan Asset Mgmt</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>350</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>7500</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>A US AI-powered market-intelligence and research platform.</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.globenewswire.com/news-release/2026/06/03/3305968/0/en/alphasense-raises-350m-at-7-5b-valuation-and-surpasses-600m-in-annual-recurring-revenue.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>InsurTech</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Honeycomb Insurance</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Zeev Ventures</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>A US AI-driven commercial-property insurance underwriter.</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>https://fortune.com/2026/06/04/honeycomb-insurance-ai-apartments-40-million/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>InsurTech</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Corgi</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>TCV</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>106</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>2600</v>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>A US full-stack commercial insurance platform.</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>https://techcrunch.com/2026/05/28/corgi-announces-106m-raise-at-2-6b-valuation-three-weeks-after-160m-series-b/</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:K7"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
     <col width="32" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="55" customWidth="1" min="10" max="10"/>
-    <col width="48" customWidth="1" min="11" max="11"/>
+    <col width="50" customWidth="1" min="10" max="10"/>
+    <col width="46" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -658,32 +1009,32 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Banking &amp; Lending Tech</t>
+          <t>Capital Markets Tech</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Capital Raise</t>
+          <t>Strategic M&amp;A</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Capchase</t>
+          <t>Funded Trading Plus</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>01 Advisors (lead)</t>
+          <t>Instant Funding</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
@@ -691,24 +1042,24 @@
       <c r="I5" s="2" t="inlineStr"/>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>A US provider of non-dilutive, revenue-based financing for B2B software firms.</t>
+          <t>A UK proprietary trading firm offering funded-trader evaluation accounts.</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>https://news.crunchbase.com/venture/fintech-capchase-b2b-bnpl-200m-debt-equity/</t>
+          <t>https://windsordrake.com/market-intelligence/transactions/funded-trading-plus-instant-funding-2026</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Capital Markets Tech</t>
+          <t>Corporate Financial Function</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -718,17 +1069,17 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Funded Trading Plus</t>
+          <t>Leapfin</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Instant Funding</t>
+          <t>Airwallex</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -736,19 +1087,19 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>A UK proprietary trading firm offering funded-trader evaluation accounts.</t>
+          <t>A US revenue-recognition and accounting-automation software provider.</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>https://windsordrake.com/market-intelligence/transactions/funded-trading-plus-instant-funding-2026</t>
+          <t>https://www.airwallex.com/global/newsroom/airwallex-acquires-leapfin-expanding-financial-lifecycle-capabilities</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Corporate Financial Function</t>
+          <t>Financial Info &amp; Analytics</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -758,7 +1109,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Capital Raise</t>
+          <t>Strategic M&amp;A</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -768,12 +1119,12 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Ramp</t>
+          <t>PEER DATA</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>ICONIQ, GIC, Ontario Teachers' (lead)</t>
+          <t>Lukka</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
@@ -781,19 +1132,19 @@
       <c r="I7" s="2" t="inlineStr"/>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>A US corporate spend-management and financial-operations platform.</t>
+          <t>A provider of data-provenance and compliance infrastructure for digital assets.</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/ramp-raises-series-f-at-44-billion-valuation-302791103.html</t>
+          <t>http://www.prnewswire.com/news-releases/lukka-acquires-peer-data-to-build-the-institutional-control-layer-for-digital-assets-and-data-commerce-302791630.html</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Corporate Financial Function</t>
+          <t>InsurTech</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -808,82 +1159,86 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Leapfin</t>
+          <t>Aggne (Aggne Global)</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Airwallex</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr"/>
+          <t>Wipro</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>28.5</v>
+      </c>
       <c r="H8" s="2" t="inlineStr"/>
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>A US revenue-recognition and accounting-automation software provider.</t>
+          <t>A US property-and-casualty insurance technology and consulting firm.</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>https://www.airwallex.com/global/newsroom/airwallex-acquires-leapfin-expanding-financial-lifecycle-capabilities</t>
+          <t>https://www.business-standard.com/amp/companies/news/wipro-raises-stake-in-insurance-tech-firm-aggne-to-80-for-28-5-million-126060102064_1.html</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Corporate Financial Function</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Capital Raise</t>
+          <t>Strategic M&amp;A</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Pivot</t>
+          <t>KUBRA (Kubra Data Transfer)</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Forestay Capital &amp; Notion Capital (lead)</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr"/>
+          <t>REPAY</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>372</v>
+      </c>
       <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>A French AI procurement and spend-management software provider.</t>
+          <t>A Canadian billing and customer-payments technology provider for utilities and government.</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2026/05/21/3299278/0/en/Pivot-Raises-40-Million-Series-B-to-Replace-Legacy-Procurement-Software-with-an-Enterprise-AI-Operating-System.html</t>
+          <t>https://investors.repay.com/news-releases/news-release-details/repay-announces-agreement-acquire-kubra</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Financial Info &amp; Analytics</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -893,22 +1248,22 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Capital Raise</t>
+          <t>Strategic M&amp;A</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>AlphaSense</t>
+          <t>Fee Navigator</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Vitruvian Partners, Accenture Ventures, J.P. Morgan Asset Mgmt (lead)</t>
+          <t>NMI</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -916,134 +1271,138 @@
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>A US AI-powered market-intelligence and research platform.</t>
+          <t>A US AI merchant-pricing intelligence provider for payments.</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2026/06/03/3305968/0/en/alphasense-raises-350m-at-7-5b-valuation-and-surpasses-600m-in-annual-recurring-revenue.html</t>
+          <t>https://www.businesswire.com/news/home/20260602447713/en/NMI-Acquires-Fee-Navigator-Adding-AI-Powered-Pricing-Intelligence-to-Its-Embedded-Payments-Platform</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Financial Info &amp; Analytics</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Strategic M&amp;A</t>
+          <t>SPAC merger (de-SPAC)</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>PEER DATA</t>
+          <t>OpenPayd</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Lukka</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr"/>
+          <t>Titan Acquisition Corp (SPAC)</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>1100</v>
+      </c>
       <c r="H11" s="2" t="inlineStr"/>
       <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>A provider of data-provenance and compliance infrastructure for digital assets.</t>
+          <t>A UK embedded-finance and payments-orchestration platform.</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>http://www.prnewswire.com/news-releases/lukka-acquires-peer-data-to-build-the-institutional-control-layer-for-digital-assets-and-data-commerce-302791630.html</t>
+          <t>https://www.globenewswire.com/news-release/2026/06/01/3304275/0/en/OpenPayd-Targets-Nasdaq-Listing-at-Unicorn-Valuation.html</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>InsurTech</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Capital Raise</t>
+          <t>Strategic M&amp;A</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Honeycomb Insurance</t>
+          <t>WonderFi</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Zeev Ventures (lead)</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr"/>
+          <t>Robinhood</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>182</v>
+      </c>
       <c r="H12" s="2" t="inlineStr"/>
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>A US AI-driven commercial-property insurance underwriter.</t>
+          <t>A Canadian operator of regulated crypto exchanges (Bitbuy and Coinsquare).</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>https://fortune.com/2026/06/04/honeycomb-insurance-ai-apartments-40-million/</t>
+          <t>https://www.newsfilecorp.com/release/299681/Robinhood-Completes-Acquisition-of-WonderFi</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>InsurTech</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Capital Raise</t>
+          <t>Strategic M&amp;A</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Corgi</t>
+          <t>Absolute Payment Solutions</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>TCV (lead)</t>
+          <t>XFolio AI</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
@@ -1051,24 +1410,24 @@
       <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>A US full-stack commercial insurance platform.</t>
+          <t>A UK Pay.UK-accredited Bacs payments service provider.</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>https://techcrunch.com/2026/05/28/corgi-announces-106m-raise-at-2-6b-valuation-three-weeks-after-160m-series-b/</t>
+          <t>https://www.fintechfutures.com/m-a/xfolio-ai-acquires-absolute-payments-solutions</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>InsurTech</t>
+          <t>Real Estate &amp; Mortgage Tech</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1078,313 +1437,35 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Aggne (Aggne Global)</t>
+          <t>Accepted Financial Corp</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Wipro</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="n">
-        <v>28.5</v>
-      </c>
+          <t>Shelter Lending Corporation</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr"/>
       <c r="H14" s="2" t="inlineStr"/>
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>A US property-and-casualty insurance technology and consulting firm.</t>
+          <t>A Western-Canada alternative mortgage lender and brokerage.</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>https://www.business-standard.com/amp/companies/news/wipro-raises-stake-in-insurance-tech-firm-aggne-to-80-for-28-5-million-126060102064_1.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Payments</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Canada</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Strategic M&amp;A</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>2026-03-30</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>KUBRA (Kubra Data Transfer)</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>REPAY</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="n">
-        <v>372</v>
-      </c>
-      <c r="H15" s="2" t="inlineStr"/>
-      <c r="I15" s="2" t="inlineStr"/>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>A Canadian billing and customer-payments technology provider for utilities and government.</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>https://investors.repay.com/news-releases/news-release-details/repay-announces-agreement-acquire-kubra</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Payments</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Strategic M&amp;A</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-02</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>Fee Navigator</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>NMI</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr"/>
-      <c r="H16" s="2" t="inlineStr"/>
-      <c r="I16" s="2" t="inlineStr"/>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>A US AI merchant-pricing intelligence provider for payments.</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>https://www.businesswire.com/news/home/20260602447713/en/NMI-Acquires-Fee-Navigator-Adding-AI-Powered-Pricing-Intelligence-to-Its-Embedded-Payments-Platform</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Payments</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>United Kingdom</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>SPAC merger (de-SPAC)</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>OpenPayd</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>Titan Acquisition Corp (SPAC)</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="n">
-        <v>1100</v>
-      </c>
-      <c r="H17" s="2" t="inlineStr"/>
-      <c r="I17" s="2" t="inlineStr"/>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>A UK embedded-finance and payments-orchestration platform.</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>https://www.globenewswire.com/news-release/2026/06/01/3304275/0/en/OpenPayd-Targets-Nasdaq-Listing-at-Unicorn-Valuation.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Payments</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Canada</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Strategic M&amp;A</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>WonderFi</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Robinhood</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="n">
-        <v>182</v>
-      </c>
-      <c r="H18" s="2" t="inlineStr"/>
-      <c r="I18" s="2" t="inlineStr"/>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>A Canadian operator of regulated crypto exchanges (Bitbuy and Coinsquare).</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>https://www.newsfilecorp.com/release/299681/Robinhood-Completes-Acquisition-of-WonderFi</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Payments</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>United Kingdom</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Strategic M&amp;A</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-02</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>Absolute Payment Solutions</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>XFolio AI</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr"/>
-      <c r="H19" s="2" t="inlineStr"/>
-      <c r="I19" s="2" t="inlineStr"/>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>A UK Pay.UK-accredited Bacs payments service provider.</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>https://www.fintechfutures.com/m-a/xfolio-ai-acquires-absolute-payments-solutions</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Real Estate &amp; Mortgage Tech</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Canada</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Strategic M&amp;A</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-20</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>Accepted Financial Corp</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>Shelter Lending Corporation</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr"/>
-      <c r="H20" s="2" t="inlineStr"/>
-      <c r="I20" s="2" t="inlineStr"/>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>A Western-Canada alternative mortgage lender and brokerage.</t>
-        </is>
-      </c>
-      <c r="K20" s="2" t="inlineStr">
-        <is>
           <t>https://www.cantechletter.com/newswires/shelter-lending-corporation-announces-acquisition-of-accepted-financial-corp-accelerating-national-growth-strategy/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K20"/>
+  <autoFilter ref="A1:K14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Apply May 30 cutoff: drop pre-May-30 deals
Growth Raises 6->3 (drop Capchase May 27, Pivot May 21, Corgi May 28).
Acquisitions 13->9 (drop Funded Trading Plus May 26, Accepted Financial
May 20, KUBRA Mar 30, and WonderFi whose deal was announced in 2025).
</commit_message>
<xml_diff>
--- a/fintech-deals-verified.xlsx
+++ b/fintech-deals-verified.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Acquisitions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Growth Raises'!$A$1:$K$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Acquisitions'!$A$1:$K$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Growth Raises'!$A$1:$K$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Acquisitions'!$A$1:$K$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -523,7 +523,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Banking &amp; Lending Tech</t>
+          <t>Corporate Financial Function</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -533,40 +533,42 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Capchase</t>
+          <t>Ramp</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>01 Advisors</t>
+          <t>ICONIQ, GIC, Ontario Teachers'</t>
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>26</v>
-      </c>
-      <c r="G2" s="2" t="inlineStr"/>
+        <v>750</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>44000</v>
+      </c>
       <c r="H2" s="2" t="inlineStr"/>
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>A US provider of non-dilutive, revenue-based financing for B2B software firms.</t>
+          <t>A US corporate spend-management and financial-operations platform.</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>https://news.crunchbase.com/venture/fintech-capchase-b2b-bnpl-200m-debt-equity/</t>
+          <t>https://www.prnewswire.com/news-releases/ramp-raises-series-f-at-44-billion-valuation-302791103.html</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Corporate Financial Function</t>
+          <t>Financial Info &amp; Analytics</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -576,62 +578,62 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Ramp</t>
+          <t>AlphaSense</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>ICONIQ, GIC, Ontario Teachers'</t>
+          <t>Vitruvian Partners, Accenture Ventures, J.P. Morgan Asset Mgmt</t>
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>750</v>
+        <v>350</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>44000</v>
+        <v>7500</v>
       </c>
       <c r="H3" s="2" t="inlineStr"/>
       <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>A US corporate spend-management and financial-operations platform.</t>
+          <t>A US AI-powered market-intelligence and research platform.</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/ramp-raises-series-f-at-44-billion-valuation-302791103.html</t>
+          <t>https://www.globenewswire.com/news-release/2026/06/03/3305968/0/en/alphasense-raises-350m-at-7-5b-valuation-and-surpasses-600m-in-annual-recurring-revenue.html</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Corporate Financial Function</t>
+          <t>InsurTech</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Pivot</t>
+          <t>Honeycomb Insurance</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Forestay Capital &amp; Notion Capital</t>
+          <t>Zeev Ventures</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
@@ -642,150 +644,17 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>A French AI procurement and spend-management software provider.</t>
+          <t>A US AI-driven commercial-property insurance underwriter.</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2026/05/21/3299278/0/en/Pivot-Raises-40-Million-Series-B-to-Replace-Legacy-Procurement-Software-with-an-Enterprise-AI-Operating-System.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Financial Info &amp; Analytics</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-03</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>AlphaSense</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Vitruvian Partners, Accenture Ventures, J.P. Morgan Asset Mgmt</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>350</v>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>7500</v>
-      </c>
-      <c r="H5" s="2" t="inlineStr"/>
-      <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>A US AI-powered market-intelligence and research platform.</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>https://www.globenewswire.com/news-release/2026/06/03/3305968/0/en/alphasense-raises-350m-at-7-5b-valuation-and-surpasses-600m-in-annual-recurring-revenue.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>InsurTech</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-04</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Honeycomb Insurance</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Zeev Ventures</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr"/>
-      <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>A US AI-driven commercial-property insurance underwriter.</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
           <t>https://fortune.com/2026/06/04/honeycomb-insurance-ai-apartments-40-million/</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>InsurTech</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Corgi</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>TCV</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>106</v>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>2600</v>
-      </c>
-      <c r="H7" s="2" t="inlineStr"/>
-      <c r="I7" s="2" t="inlineStr"/>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>A US full-stack commercial insurance platform.</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>https://techcrunch.com/2026/05/28/corgi-announces-106m-raise-at-2-6b-valuation-three-weeks-after-160m-series-b/</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:K7"/>
+  <autoFilter ref="A1:K4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -796,7 +665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1009,12 +878,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Capital Markets Tech</t>
+          <t>Corporate Financial Function</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -1024,17 +893,17 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Funded Trading Plus</t>
+          <t>Leapfin</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Instant Funding</t>
+          <t>Airwallex</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
@@ -1042,19 +911,19 @@
       <c r="I5" s="2" t="inlineStr"/>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>A UK proprietary trading firm offering funded-trader evaluation accounts.</t>
+          <t>A US revenue-recognition and accounting-automation software provider.</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>https://windsordrake.com/market-intelligence/transactions/funded-trading-plus-instant-funding-2026</t>
+          <t>https://www.airwallex.com/global/newsroom/airwallex-acquires-leapfin-expanding-financial-lifecycle-capabilities</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Corporate Financial Function</t>
+          <t>Financial Info &amp; Analytics</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -1074,12 +943,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Leapfin</t>
+          <t>PEER DATA</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Airwallex</t>
+          <t>Lukka</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -1087,19 +956,19 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>A US revenue-recognition and accounting-automation software provider.</t>
+          <t>A provider of data-provenance and compliance infrastructure for digital assets.</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>https://www.airwallex.com/global/newsroom/airwallex-acquires-leapfin-expanding-financial-lifecycle-capabilities</t>
+          <t>http://www.prnewswire.com/news-releases/lukka-acquires-peer-data-to-build-the-institutional-control-layer-for-digital-assets-and-data-commerce-302791630.html</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Financial Info &amp; Analytics</t>
+          <t>InsurTech</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -1114,37 +983,39 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>PEER DATA</t>
+          <t>Aggne (Aggne Global)</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Lukka</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr"/>
+          <t>Wipro</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>28.5</v>
+      </c>
       <c r="H7" s="2" t="inlineStr"/>
       <c r="I7" s="2" t="inlineStr"/>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>A provider of data-provenance and compliance infrastructure for digital assets.</t>
+          <t>A US property-and-casualty insurance technology and consulting firm.</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>http://www.prnewswire.com/news-releases/lukka-acquires-peer-data-to-build-the-institutional-control-layer-for-digital-assets-and-data-commerce-302791630.html</t>
+          <t>https://www.business-standard.com/amp/companies/news/wipro-raises-stake-in-insurance-tech-firm-aggne-to-80-for-28-5-million-126060102064_1.html</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>InsurTech</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1159,32 +1030,30 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Aggne (Aggne Global)</t>
+          <t>Fee Navigator</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Wipro</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="n">
-        <v>28.5</v>
-      </c>
+          <t>NMI</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr"/>
       <c r="H8" s="2" t="inlineStr"/>
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>A US property-and-casualty insurance technology and consulting firm.</t>
+          <t>A US AI merchant-pricing intelligence provider for payments.</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>https://www.business-standard.com/amp/companies/news/wipro-raises-stake-in-insurance-tech-firm-aggne-to-80-for-28-5-million-126060102064_1.html</t>
+          <t>https://www.businesswire.com/news/home/20260602447713/en/NMI-Acquires-Fee-Navigator-Adding-AI-Powered-Pricing-Intelligence-to-Its-Embedded-Payments-Platform</t>
         </is>
       </c>
     </row>
@@ -1196,42 +1065,42 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Strategic M&amp;A</t>
+          <t>SPAC merger (de-SPAC)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>KUBRA (Kubra Data Transfer)</t>
+          <t>OpenPayd</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>REPAY</t>
+          <t>Titan Acquisition Corp (SPAC)</t>
         </is>
       </c>
       <c r="G9" s="2" t="n">
-        <v>372</v>
+        <v>1100</v>
       </c>
       <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>A Canadian billing and customer-payments technology provider for utilities and government.</t>
+          <t>A UK embedded-finance and payments-orchestration platform.</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>https://investors.repay.com/news-releases/news-release-details/repay-announces-agreement-acquire-kubra</t>
+          <t>https://www.globenewswire.com/news-release/2026/06/01/3304275/0/en/OpenPayd-Targets-Nasdaq-Listing-at-Unicorn-Valuation.html</t>
         </is>
       </c>
     </row>
@@ -1243,7 +1112,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1258,12 +1127,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Fee Navigator</t>
+          <t>Absolute Payment Solutions</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>NMI</t>
+          <t>XFolio AI</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -1271,201 +1140,17 @@
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>A US AI merchant-pricing intelligence provider for payments.</t>
+          <t>A UK Pay.UK-accredited Bacs payments service provider.</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>https://www.businesswire.com/news/home/20260602447713/en/NMI-Acquires-Fee-Navigator-Adding-AI-Powered-Pricing-Intelligence-to-Its-Embedded-Payments-Platform</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Payments</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>United Kingdom</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>SPAC merger (de-SPAC)</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>OpenPayd</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>Titan Acquisition Corp (SPAC)</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="n">
-        <v>1100</v>
-      </c>
-      <c r="H11" s="2" t="inlineStr"/>
-      <c r="I11" s="2" t="inlineStr"/>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>A UK embedded-finance and payments-orchestration platform.</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>https://www.globenewswire.com/news-release/2026/06/01/3304275/0/en/OpenPayd-Targets-Nasdaq-Listing-at-Unicorn-Valuation.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Payments</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Canada</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Strategic M&amp;A</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>WonderFi</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>Robinhood</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="n">
-        <v>182</v>
-      </c>
-      <c r="H12" s="2" t="inlineStr"/>
-      <c r="I12" s="2" t="inlineStr"/>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>A Canadian operator of regulated crypto exchanges (Bitbuy and Coinsquare).</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>https://www.newsfilecorp.com/release/299681/Robinhood-Completes-Acquisition-of-WonderFi</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Payments</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>United Kingdom</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Strategic M&amp;A</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-02</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Absolute Payment Solutions</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>XFolio AI</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr"/>
-      <c r="I13" s="2" t="inlineStr"/>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>A UK Pay.UK-accredited Bacs payments service provider.</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
           <t>https://www.fintechfutures.com/m-a/xfolio-ai-acquires-absolute-payments-solutions</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Real Estate &amp; Mortgage Tech</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Canada</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Strategic M&amp;A</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-20</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>Accepted Financial Corp</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>Shelter Lending Corporation</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr"/>
-      <c r="H14" s="2" t="inlineStr"/>
-      <c r="I14" s="2" t="inlineStr"/>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>A Western-Canada alternative mortgage lender and brokerage.</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>https://www.cantechletter.com/newswires/shelter-lending-corporation-announces-acquisition-of-accepted-financial-corp-accelerating-national-growth-strategy/</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:K14"/>
+  <autoFilter ref="A1:K10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>